<commit_message>
chore: atualizar planilha modelo
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/modelo.xlsx
+++ b/public/modelo.xlsx
@@ -452,4 +452,251 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100BA43650AF5E7044186EA8321ACFAC10A" ma:contentTypeVersion="13" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1066ad7483069042308fc283768ecd85">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a3b453bc-c24f-41be-b740-a4183b313a53" xmlns:ns3="fb698544-796c-4388-a554-e2b8dc72b864" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b30ffee1ad420e8b8425cffe44ae7bcf" ns2:_="" ns3:_="">
+    <xsd:import namespace="a3b453bc-c24f-41be-b740-a4183b313a53"/>
+    <xsd:import namespace="fb698544-796c-4388-a554-e2b8dc72b864"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:Raz_x00e3_o_x0020_Social" minOccurs="0"/>
+                <xsd:element ref="ns2:CNPJ" minOccurs="0"/>
+                <xsd:element ref="ns2:Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a3b453bc-c24f-41be-b740-a4183b313a53" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Raz_x00e3_o_x0020_Social" ma:index="11" nillable="true" ma:displayName="Razão Social" ma:internalName="Raz_x00e3_o_x0020_Social">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="CNPJ" ma:index="12" nillable="true" ma:displayName="CNPJ" ma:internalName="CNPJ">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio" ma:index="13" nillable="true" ma:displayName="Qual é a tipologia do negócio" ma:format="Dropdown" ma:internalName="Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Choice">
+          <xsd:enumeration value="Custodiante"/>
+          <xsd:enumeration value="Intermediária"/>
+          <xsd:enumeration value="Corretora"/>
+          <xsd:enumeration value="Instituição regulada pelo BACEN"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e6b9a89d-d12a-4c50-a0c9-d06604afc248" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="20" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="fb698544-796c-4388-a554-e2b8dc72b864" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{cbb0f04e-9b81-4396-90de-a59917bee501}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="fb698544-796c-4388-a554-e2b8dc72b864">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <CNPJ xmlns="a3b453bc-c24f-41be-b740-a4183b313a53" xsi:nil="true"/>
+    <TaxCatchAll xmlns="fb698544-796c-4388-a554-e2b8dc72b864" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a3b453bc-c24f-41be-b740-a4183b313a53">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio xmlns="a3b453bc-c24f-41be-b740-a4183b313a53" xsi:nil="true"/>
+    <Raz_x00e3_o_x0020_Social xmlns="a3b453bc-c24f-41be-b740-a4183b313a53" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F2C034C-1E0A-4C29-A1C0-2B386705CC1C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5993B8E6-431E-4D1B-9961-B5DE131E9627}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{636FBD9E-FA68-4A7E-B43A-DB9E25F052C8}"/>
 </file>
</xml_diff>

<commit_message>
chore: atualizar planilha modelo com colunas atuais
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/modelo.xlsx
+++ b/public/modelo.xlsx
@@ -31,28 +31,43 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <b/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill patternType="none">
+        <bgColor/>
+      </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -61,13 +76,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -399,51 +419,51 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
   <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="17.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
+      <c r="A1" s="3" t="str">
         <v>ticker</v>
       </c>
-      <c r="B1" t="str">
+      <c r="B1" s="3" t="str">
         <v>quantidade</v>
       </c>
-      <c r="C1" t="str">
+      <c r="C1" s="3" t="str">
         <v>valor_declarado</v>
       </c>
-      <c r="D1" t="str">
+      <c r="D1" s="3" t="str">
         <v>data_base</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2" s="2" t="str">
         <v>BTC</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>2.5</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="2">
         <v>750000</v>
       </c>
-      <c r="D2" t="str">
+      <c r="D2" s="2" t="str">
         <v>2024-12-31</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3" s="2" t="str">
         <v>ETH</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>10</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>200000</v>
       </c>
-      <c r="D3" t="str">
+      <c r="D3" s="2" t="str">
         <v>2024-12-31</v>
       </c>
     </row>
@@ -452,251 +472,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100BA43650AF5E7044186EA8321ACFAC10A" ma:contentTypeVersion="13" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1066ad7483069042308fc283768ecd85">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a3b453bc-c24f-41be-b740-a4183b313a53" xmlns:ns3="fb698544-796c-4388-a554-e2b8dc72b864" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b30ffee1ad420e8b8425cffe44ae7bcf" ns2:_="" ns3:_="">
-    <xsd:import namespace="a3b453bc-c24f-41be-b740-a4183b313a53"/>
-    <xsd:import namespace="fb698544-796c-4388-a554-e2b8dc72b864"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:Raz_x00e3_o_x0020_Social" minOccurs="0"/>
-                <xsd:element ref="ns2:CNPJ" minOccurs="0"/>
-                <xsd:element ref="ns2:Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a3b453bc-c24f-41be-b740-a4183b313a53" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Raz_x00e3_o_x0020_Social" ma:index="11" nillable="true" ma:displayName="Razão Social" ma:internalName="Raz_x00e3_o_x0020_Social">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="CNPJ" ma:index="12" nillable="true" ma:displayName="CNPJ" ma:internalName="CNPJ">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio" ma:index="13" nillable="true" ma:displayName="Qual é a tipologia do negócio" ma:format="Dropdown" ma:internalName="Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Choice">
-          <xsd:enumeration value="Custodiante"/>
-          <xsd:enumeration value="Intermediária"/>
-          <xsd:enumeration value="Corretora"/>
-          <xsd:enumeration value="Instituição regulada pelo BACEN"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="18" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e6b9a89d-d12a-4c50-a0c9-d06604afc248" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="20" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="fb698544-796c-4388-a554-e2b8dc72b864" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="19" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{cbb0f04e-9b81-4396-90de-a59917bee501}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="fb698544-796c-4388-a554-e2b8dc72b864">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <CNPJ xmlns="a3b453bc-c24f-41be-b740-a4183b313a53" xsi:nil="true"/>
-    <TaxCatchAll xmlns="fb698544-796c-4388-a554-e2b8dc72b864" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a3b453bc-c24f-41be-b740-a4183b313a53">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Qual_x0020__x00e9__x0020_a_x0020_tipologia_x0020_do_x0020_neg_x00f3_cio xmlns="a3b453bc-c24f-41be-b740-a4183b313a53" xsi:nil="true"/>
-    <Raz_x00e3_o_x0020_Social xmlns="a3b453bc-c24f-41be-b740-a4183b313a53" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F2C034C-1E0A-4C29-A1C0-2B386705CC1C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5993B8E6-431E-4D1B-9961-B5DE131E9627}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{636FBD9E-FA68-4A7E-B43A-DB9E25F052C8}"/>
 </file>
</xml_diff>